<commit_message>
Procesteknolog: hands-on er nu en Excel-opgave med egne formler
Fanen Opgave i datasættet med tomme kolonner og inputceller. Opgaveark (Bilag F)
under Materialer, nyt slide med trinnene, Din tur og pointe omskrevet.
Facit-ark med formlerne ligger i undervisningsplanens mappe.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015YJpkwAMXruZRjbkCwcfYy
</commit_message>
<xml_diff>
--- a/public/p/proces/filer/Procesteknolog_Fjordtoerreriet_2026.xlsx
+++ b/public/p/proces/filer/Procesteknolog_Fjordtoerreriet_2026.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fugtlog" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Luft" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operatørnoter" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opgave" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +56,19 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="006E6E73"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +78,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F2430"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003D74FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -97,6 +119,14 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -538,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -601,28 +631,35 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Opgave. De 14 batches med tomme kolonner til jeres egne formler. Se opgavearket fra timen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Massebalancen</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Tørstoffet er det samme før og efter tørring. Tørstof = ind x (1 - vandindhold ind). Masse ud = tørstof / (1 - vandindhold ud). Vand fjernet = ind - masse ud.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Sådan bruger du filen</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Upload filen til Claude, ChatGPT eller Copilot, og brug promptkortet fra timen. Eller arbejd direkte i Excel.</t>
         </is>
@@ -30243,4 +30280,888 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Batchnr.</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Vare</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Sort</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Planlager</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Slut</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Ind (kg)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Vandindhold ind</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Vandindhold ud</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Ud, brovægt (kg)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Blæser og varme (kWh)</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>Timer</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="inlineStr">
+        <is>
+          <t>Tørstof (kg)</t>
+        </is>
+      </c>
+      <c r="N1" s="11" t="inlineStr">
+        <is>
+          <t>Masse ud (kg)</t>
+        </is>
+      </c>
+      <c r="O1" s="11" t="inlineStr">
+        <is>
+          <t>Vand fjernet (kg)</t>
+        </is>
+      </c>
+      <c r="P1" s="11" t="inlineStr">
+        <is>
+          <t>Vand pr. time (kg)</t>
+        </is>
+      </c>
+      <c r="Q1" s="11" t="inlineStr">
+        <is>
+          <t>Tørstof ved slut</t>
+        </is>
+      </c>
+      <c r="R1" s="11" t="inlineStr">
+        <is>
+          <t>Tørstof, hvis ekstra vand fjernes</t>
+        </is>
+      </c>
+      <c r="S1" s="11" t="inlineStr">
+        <is>
+          <t>Difference til brovægt</t>
+        </is>
+      </c>
+      <c r="T1" s="11" t="inlineStr">
+        <is>
+          <t>Tjek</t>
+        </is>
+      </c>
+      <c r="V1" s="12" t="inlineStr">
+        <is>
+          <t>Ekstra vand fjernet (kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>T-01</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Vårbyg</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>PL1</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>46244.33333333334</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>46248.33333333334</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>212000</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>202130</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>2960</v>
+      </c>
+      <c r="L2" s="13" t="n"/>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="n"/>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="9" t="n"/>
+      <c r="Q2" s="8" t="n"/>
+      <c r="R2" s="8" t="n"/>
+      <c r="S2" s="8" t="n"/>
+      <c r="T2" s="5" t="n"/>
+      <c r="V2" s="14" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>T-02</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Krydderurter</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Dild</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>PL3</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>46245.25</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>46247.08333333334</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>84000</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>72170</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>2490</v>
+      </c>
+      <c r="L3" s="13" t="n"/>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="7" t="n"/>
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="9" t="n"/>
+      <c r="Q3" s="8" t="n"/>
+      <c r="R3" s="8" t="n"/>
+      <c r="S3" s="8" t="n"/>
+      <c r="T3" s="5" t="n"/>
+      <c r="V3" s="12" t="inlineStr">
+        <is>
+          <t>Grænse for brovægt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>T-03</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Vinterhvede</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>PL2</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>46248.41666666666</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>46254.91666666666</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>268000</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>249450</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>4700</v>
+      </c>
+      <c r="L4" s="13" t="n"/>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="7" t="n"/>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="9" t="n"/>
+      <c r="Q4" s="8" t="n"/>
+      <c r="R4" s="8" t="n"/>
+      <c r="S4" s="8" t="n"/>
+      <c r="T4" s="5" t="n"/>
+      <c r="V4" s="15" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>T-04</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Vinterhvede</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>PL1</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>46249.29166666666</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>46254.79166666666</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>240000</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>225650</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L5" s="13" t="n"/>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="7" t="n"/>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="9" t="n"/>
+      <c r="Q5" s="8" t="n"/>
+      <c r="R5" s="8" t="n"/>
+      <c r="S5" s="8" t="n"/>
+      <c r="T5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>T-05</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Krydderurter</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Persille</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>PL3</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>46251.25</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>46253.58333333334</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>102000</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>85780</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>3090</v>
+      </c>
+      <c r="L6" s="13" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="9" t="n"/>
+      <c r="Q6" s="8" t="n"/>
+      <c r="R6" s="8" t="n"/>
+      <c r="S6" s="8" t="n"/>
+      <c r="T6" s="5" t="n"/>
+      <c r="V6" s="16" t="inlineStr">
+        <is>
+          <t>Gule celler er input. Blå kolonner udfylder I med formler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>T-06</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Tang</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Sukkertang</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>PL2</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>46256.375</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>46260.875</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>276000</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>245880</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>3210</v>
+      </c>
+      <c r="L7" s="13" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="9" t="n"/>
+      <c r="Q7" s="8" t="n"/>
+      <c r="R7" s="8" t="n"/>
+      <c r="S7" s="8" t="n"/>
+      <c r="T7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>T-07</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Vinterhvede</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>PL1</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>46258.25</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>46263.58333333334</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>230000</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>215210</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>3770</v>
+      </c>
+      <c r="L8" s="13" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="9" t="n"/>
+      <c r="Q8" s="8" t="n"/>
+      <c r="R8" s="8" t="n"/>
+      <c r="S8" s="8" t="n"/>
+      <c r="T8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>T-08</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Vårbyg</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>PL1</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>46265.33333333334</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>46269.5</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>198000</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0.147</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>184150</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>3080</v>
+      </c>
+      <c r="L9" s="13" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="9" t="n"/>
+      <c r="Q9" s="8" t="n"/>
+      <c r="R9" s="8" t="n"/>
+      <c r="S9" s="8" t="n"/>
+      <c r="T9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>T-09</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Tang</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Sukkertang</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>PL2</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>46266.33333333334</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>46271.16666666666</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>290000</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>258080</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>3530</v>
+      </c>
+      <c r="L10" s="13" t="n"/>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="9" t="n"/>
+      <c r="Q10" s="8" t="n"/>
+      <c r="R10" s="8" t="n"/>
+      <c r="S10" s="8" t="n"/>
+      <c r="T10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>T-10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Krydderurter</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Timian</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>PL3</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>46268.29166666666</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>46270.79166666666</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>96000</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>81190</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>3450</v>
+      </c>
+      <c r="L11" s="13" t="n"/>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="7" t="n"/>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="9" t="n"/>
+      <c r="Q11" s="8" t="n"/>
+      <c r="R11" s="8" t="n"/>
+      <c r="S11" s="8" t="n"/>
+      <c r="T11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>T-11</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Krydderurter</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Persille</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>PL3</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>46273.25</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>46275.41666666666</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>110000</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>93370</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>2910</v>
+      </c>
+      <c r="L12" s="13" t="n"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="9" t="n"/>
+      <c r="Q12" s="8" t="n"/>
+      <c r="R12" s="8" t="n"/>
+      <c r="S12" s="8" t="n"/>
+      <c r="T12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>T-12</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Krydderurter</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Dild</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>PL3</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>46276.25</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>46279.25</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>88000</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>73440</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>4140</v>
+      </c>
+      <c r="L13" s="13" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="9" t="n"/>
+      <c r="Q13" s="8" t="n"/>
+      <c r="R13" s="8" t="n"/>
+      <c r="S13" s="8" t="n"/>
+      <c r="T13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>T-13</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Vårbyg</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>PL1</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>46284.33333333334</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>205000</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>194750</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>3430</v>
+      </c>
+      <c r="L14" s="13" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="9" t="n"/>
+      <c r="Q14" s="8" t="n"/>
+      <c r="R14" s="8" t="n"/>
+      <c r="S14" s="8" t="n"/>
+      <c r="T14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>T-14</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Korn</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Havre</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>PL2</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>46295.33333333334</v>
+      </c>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="7" t="n">
+        <v>236000</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n">
+        <v>6420</v>
+      </c>
+      <c r="L15" s="13" t="n"/>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="n"/>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="9" t="n"/>
+      <c r="Q15" s="8" t="n"/>
+      <c r="R15" s="8" t="n"/>
+      <c r="S15" s="8" t="n"/>
+      <c r="T15" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Procesteknolog: mindre opgave med ChatGPT i Excel
Fanen Opgave har nu kun de tre spørgsmål fra Opgave 13 for 13 batches.
Opgavearket beder dem åbne ChatGPT i Excel, bede om formlerne og tjekke
T-07, T-09 og T-11 mod deres egen udregning. Slides og plan fulgt med.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015YJpkwAMXruZRjbkCwcfYy
</commit_message>
<xml_diff>
--- a/public/p/proces/filer/Procesteknolog_Fjordtoerreriet_2026.xlsx
+++ b/public/p/proces/filer/Procesteknolog_Fjordtoerreriet_2026.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,17 +58,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
       <color rgb="006E6E73"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -85,11 +80,6 @@
         <fgColor rgb="003D74FF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF4CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -103,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,9 +114,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -633,7 +620,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Opgave. De 14 batches med tomme kolonner til jeres egne formler. Se opgavearket fra timen.</t>
+          <t>Opgave. De 13 afsluttede batches med tre tomme kolonner til de tre spørgsmål fra Opgave 13. Se opgavearket fra timen.</t>
         </is>
       </c>
     </row>
@@ -30288,30 +30275,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -30327,97 +30303,47 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Sort</t>
+          <t>Ind (kg)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Planlager</t>
+          <t>Timer</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>Vandindhold ind</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Slut</t>
+          <t>Vandindhold ud</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Ind (kg)</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Vandindhold ind</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>Vandindhold ud</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Ud, brovægt (kg)</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>Blæser og varme (kWh)</t>
-        </is>
-      </c>
-      <c r="L1" s="11" t="inlineStr">
-        <is>
-          <t>Timer</t>
-        </is>
-      </c>
-      <c r="M1" s="11" t="inlineStr">
-        <is>
-          <t>Tørstof (kg)</t>
-        </is>
-      </c>
-      <c r="N1" s="11" t="inlineStr">
-        <is>
-          <t>Masse ud (kg)</t>
-        </is>
-      </c>
-      <c r="O1" s="11" t="inlineStr">
+          <t>Ekstra vand fjernet (kg)</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Vand fjernet (kg)</t>
         </is>
       </c>
-      <c r="P1" s="11" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Vand pr. time (kg)</t>
         </is>
       </c>
-      <c r="Q1" s="11" t="inlineStr">
-        <is>
-          <t>Tørstof ved slut</t>
-        </is>
-      </c>
-      <c r="R1" s="11" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Tørstof, hvis ekstra vand fjernes</t>
         </is>
       </c>
-      <c r="S1" s="11" t="inlineStr">
-        <is>
-          <t>Difference til brovægt</t>
-        </is>
-      </c>
-      <c r="T1" s="11" t="inlineStr">
-        <is>
-          <t>Tjek</t>
-        </is>
-      </c>
-      <c r="V1" s="12" t="inlineStr">
-        <is>
-          <t>Ekstra vand fjernet (kg)</t>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>De blå kolonner H, I og J udfylder I. Se opgavearket fra timen.</t>
         </is>
       </c>
     </row>
@@ -30432,49 +30358,24 @@
           <t>Korn</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Vårbyg</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>PL1</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>46244.33333333334</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>46248.33333333334</v>
+      <c r="C2" s="7" t="n">
+        <v>212000</v>
+      </c>
+      <c r="D2" s="13" t="n">
+        <v>96</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>0.148</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>212000</v>
-      </c>
-      <c r="H2" s="8" t="n">
-        <v>0.184</v>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>0.148</v>
-      </c>
-      <c r="J2" s="7" t="n">
-        <v>202130</v>
-      </c>
-      <c r="K2" s="7" t="n">
-        <v>2960</v>
-      </c>
-      <c r="L2" s="13" t="n"/>
-      <c r="M2" s="7" t="n"/>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="9" t="n"/>
-      <c r="Q2" s="8" t="n"/>
-      <c r="R2" s="8" t="n"/>
-      <c r="S2" s="8" t="n"/>
-      <c r="T2" s="5" t="n"/>
-      <c r="V2" s="14" t="n">
         <v>1500</v>
       </c>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="9" t="n"/>
+      <c r="J2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -30487,51 +30388,24 @@
           <t>Krydderurter</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Dild</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>PL3</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>46245.25</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>46247.08333333334</v>
+      <c r="C3" s="7" t="n">
+        <v>84000</v>
+      </c>
+      <c r="D3" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>0.118</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>84000</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>0.241</v>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0.118</v>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>72170</v>
-      </c>
-      <c r="K3" s="7" t="n">
-        <v>2490</v>
-      </c>
-      <c r="L3" s="13" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="9" t="n"/>
-      <c r="Q3" s="8" t="n"/>
-      <c r="R3" s="8" t="n"/>
-      <c r="S3" s="8" t="n"/>
-      <c r="T3" s="5" t="n"/>
-      <c r="V3" s="12" t="inlineStr">
-        <is>
-          <t>Grænse for brovægt</t>
-        </is>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="9" t="n"/>
+      <c r="J3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -30544,49 +30418,24 @@
           <t>Korn</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Vinterhvede</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>PL2</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>46248.41666666666</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>46254.91666666666</v>
+      <c r="C4" s="7" t="n">
+        <v>268000</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>156</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.153</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>268000</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0.153</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>249450</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>4700</v>
-      </c>
-      <c r="L4" s="13" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="9" t="n"/>
-      <c r="Q4" s="8" t="n"/>
-      <c r="R4" s="8" t="n"/>
-      <c r="S4" s="8" t="n"/>
-      <c r="T4" s="5" t="n"/>
-      <c r="V4" s="15" t="n">
-        <v>0.01</v>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="9" t="n"/>
+      <c r="J4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -30599,46 +30448,24 @@
           <t>Korn</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Vinterhvede</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>PL1</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>46249.29166666666</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>46254.79166666666</v>
+      <c r="C5" s="7" t="n">
+        <v>240000</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>132</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0.149</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>240000</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>0.196</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0.149</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>225650</v>
-      </c>
-      <c r="K5" s="7" t="n">
-        <v>4000</v>
-      </c>
-      <c r="L5" s="13" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="9" t="n"/>
-      <c r="Q5" s="8" t="n"/>
-      <c r="R5" s="8" t="n"/>
-      <c r="S5" s="8" t="n"/>
-      <c r="T5" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -30651,51 +30478,24 @@
           <t>Krydderurter</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Persille</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>PL3</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>46251.25</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>46253.58333333334</v>
+      <c r="C6" s="7" t="n">
+        <v>102000</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>56</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.122</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>102000</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>0.258</v>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>85780</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>3090</v>
-      </c>
-      <c r="L6" s="13" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="9" t="n"/>
-      <c r="Q6" s="8" t="n"/>
-      <c r="R6" s="8" t="n"/>
-      <c r="S6" s="8" t="n"/>
-      <c r="T6" s="5" t="n"/>
-      <c r="V6" s="16" t="inlineStr">
-        <is>
-          <t>Gule celler er input. Blå kolonner udfylder I med formler.</t>
-        </is>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -30708,46 +30508,24 @@
           <t>Tang</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Sukkertang</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>PL2</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>46256.375</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>46260.875</v>
+      <c r="C7" s="7" t="n">
+        <v>276000</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>108</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0.158</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>276000</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>0.246</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0.158</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>245880</v>
-      </c>
-      <c r="K7" s="7" t="n">
-        <v>3210</v>
-      </c>
-      <c r="L7" s="13" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="9" t="n"/>
-      <c r="Q7" s="8" t="n"/>
-      <c r="R7" s="8" t="n"/>
-      <c r="S7" s="8" t="n"/>
-      <c r="T7" s="5" t="n"/>
+        <v>1250</v>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -30760,46 +30538,24 @@
           <t>Korn</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Vinterhvede</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>PL1</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>46258.25</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>46263.58333333334</v>
+      <c r="C8" s="7" t="n">
+        <v>230000</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>128</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.151</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>230000</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>0.202</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>0.151</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>215210</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>3770</v>
-      </c>
-      <c r="L8" s="13" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="9" t="n"/>
-      <c r="Q8" s="8" t="n"/>
-      <c r="R8" s="8" t="n"/>
-      <c r="S8" s="8" t="n"/>
-      <c r="T8" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -30812,46 +30568,24 @@
           <t>Korn</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Vårbyg</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>PL1</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>46265.33333333334</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>46269.5</v>
+      <c r="C9" s="7" t="n">
+        <v>198000</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0.147</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>198000</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>0.147</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>184150</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>3080</v>
-      </c>
-      <c r="L9" s="13" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="9" t="n"/>
-      <c r="Q9" s="8" t="n"/>
-      <c r="R9" s="8" t="n"/>
-      <c r="S9" s="8" t="n"/>
-      <c r="T9" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -30864,46 +30598,24 @@
           <t>Tang</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Sukkertang</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>PL2</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>46266.33333333334</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>46271.16666666666</v>
+      <c r="C10" s="7" t="n">
+        <v>290000</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>116</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0.161</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>290000</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>0.161</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>258080</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>3530</v>
-      </c>
-      <c r="L10" s="13" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="9" t="n"/>
-      <c r="Q10" s="8" t="n"/>
-      <c r="R10" s="8" t="n"/>
-      <c r="S10" s="8" t="n"/>
-      <c r="T10" s="5" t="n"/>
+        <v>1250</v>
+      </c>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -30916,46 +30628,24 @@
           <t>Krydderurter</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Timian</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>PL3</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>46268.29166666666</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>46270.79166666666</v>
+      <c r="C11" s="7" t="n">
+        <v>96000</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0.115</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>96000</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>0.234</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>81190</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>3450</v>
-      </c>
-      <c r="L11" s="13" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="9" t="n"/>
-      <c r="Q11" s="8" t="n"/>
-      <c r="R11" s="8" t="n"/>
-      <c r="S11" s="8" t="n"/>
-      <c r="T11" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -30968,46 +30658,24 @@
           <t>Krydderurter</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Persille</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>PL3</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>46273.25</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>46275.41666666666</v>
+      <c r="C12" s="7" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>52</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0.121</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>110000</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>93370</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>2910</v>
-      </c>
-      <c r="L12" s="13" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="9" t="n"/>
-      <c r="Q12" s="8" t="n"/>
-      <c r="R12" s="8" t="n"/>
-      <c r="S12" s="8" t="n"/>
-      <c r="T12" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -31020,46 +30688,24 @@
           <t>Krydderurter</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Dild</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>PL3</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>46276.25</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>46279.25</v>
+      <c r="C13" s="7" t="n">
+        <v>88000</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>0.092</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>88000</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>0.092</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>73440</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>4140</v>
-      </c>
-      <c r="L13" s="13" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="9" t="n"/>
-      <c r="Q13" s="8" t="n"/>
-      <c r="R13" s="8" t="n"/>
-      <c r="S13" s="8" t="n"/>
-      <c r="T13" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -31072,94 +30718,24 @@
           <t>Korn</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Vårbyg</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>PL1</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>46284.33333333334</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>46289</v>
+      <c r="C14" s="7" t="n">
+        <v>205000</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>112</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>0.15</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>205000</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>0.191</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>194750</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>3430</v>
-      </c>
-      <c r="L14" s="13" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="9" t="n"/>
-      <c r="Q14" s="8" t="n"/>
-      <c r="R14" s="8" t="n"/>
-      <c r="S14" s="8" t="n"/>
-      <c r="T14" s="5" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>T-14</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Korn</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Havre</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>PL2</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>46295.33333333334</v>
-      </c>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="7" t="n">
-        <v>236000</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>0.208</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n">
-        <v>6420</v>
-      </c>
-      <c r="L15" s="13" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="9" t="n"/>
-      <c r="Q15" s="8" t="n"/>
-      <c r="R15" s="8" t="n"/>
-      <c r="S15" s="8" t="n"/>
-      <c r="T15" s="5" t="n"/>
+        <v>1500</v>
+      </c>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>